<commit_message>
EQA criterion: pass above 90% (assessed only in months EQA was run; others ND)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NCemeHN95tB9Q4N37Akmn
</commit_message>
<xml_diff>
--- a/data/POCT_KPI_Database.xlsx
+++ b/data/POCT_KPI_Database.xlsx
@@ -93928,7 +93928,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>มากกว่าร้อยละ 95 ของเครื่องตรวจทั้งหมด</t>
+          <t>มากกว่าร้อยละ 90 ของเครื่องตรวจที่เข้าร่วม (ประเมินเฉพาะเดือนที่มีการทำ EQA — เดือนที่ไม่ได้ทำใส่ ND)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -93943,7 +93943,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -93985,7 +93985,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>มากกว่าร้อยละ 95 ของเครื่องตรวจทั้งหมด</t>
+          <t>มากกว่าร้อยละ 90 ของเครื่องตรวจที่เข้าร่วม (ประเมินเฉพาะเดือนที่มีการทำ EQA — เดือนที่ไม่ได้ทำใส่ ND)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -94004,7 +94004,7 @@
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Revert EQA criterion change: 95% was correct
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NCemeHN95tB9Q4N37Akmn
</commit_message>
<xml_diff>
--- a/data/POCT_KPI_Database.xlsx
+++ b/data/POCT_KPI_Database.xlsx
@@ -93928,7 +93928,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>มากกว่าร้อยละ 90 ของเครื่องตรวจที่เข้าร่วม (ประเมินเฉพาะเดือนที่มีการทำ EQA — เดือนที่ไม่ได้ทำใส่ ND)</t>
+          <t>มากกว่าร้อยละ 95 ของเครื่องตรวจทั้งหมด</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -93943,7 +93943,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -93985,7 +93985,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>มากกว่าร้อยละ 90 ของเครื่องตรวจที่เข้าร่วม (ประเมินเฉพาะเดือนที่มีการทำ EQA — เดือนที่ไม่ได้ทำใส่ ND)</t>
+          <t>มากกว่าร้อยละ 95 ของเครื่องตรวจทั้งหมด</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -94004,7 +94004,7 @@
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>

</xml_diff>